<commit_message>
Added Prepare Payroll Module Test scenarios and Find page functions test scenarios
Added Prepare Payroll Module Test scenarios, Find page functions test scenarios and Fixed failed Leave Module Test scenarios
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -1225,7 +1225,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.72380952380952" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="4" max="4" width="10.8571428571429"/>
+    <col min="4" max="4" width="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1253,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="3">
-        <v>45771</v>
+        <v>45801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stabilized Test Script for Employee Master, Employee Adjustment, Leave and Leave Adjustment Modules.
Stabilized Test Script for Employee Master, Employee Adjustment, Leave and Leave Adjustment Modules.
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
-    <sheet name="LeaveTemplate" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>CL</t>
+  </si>
+  <si>
+    <t>21-10-2025</t>
   </si>
 </sst>
 </file>
@@ -697,7 +700,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -1223,9 +1226,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="8.72380952380952" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="4" max="4" width="13"/>
+    <col min="4" max="4" width="13.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1252,8 +1255,8 @@
       <c r="C2" s="2">
         <v>1</v>
       </c>
-      <c r="D2" s="3">
-        <v>45801</v>
+      <c r="D2" t="s" s="0">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Failed Scenarios and Stabilized Script for Process Payroll Scenario
Fixed Failed Scenarios and Stabilized Script for Process Payroll Scenario
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -48,6 +48,12 @@
   </si>
   <si>
     <t>21-10-2025</t>
+  </si>
+  <si>
+    <t>2025-11-01</t>
+  </si>
+  <si>
+    <t>2025-10-27</t>
   </si>
 </sst>
 </file>
@@ -1256,7 +1262,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Employee Master, Attendance Leave, Payroll and  and Bill of Materials Test script
Fixed Employee Master, Attendance Leave, Payroll and  and Bill of Materials Test script
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>2025-10-27</t>
+  </si>
+  <si>
+    <t>2025-11-17</t>
   </si>
 </sst>
 </file>
@@ -1262,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Production Order test scenarios and Leave Adjustment scenarios
Fixed Production Order test scenarios and Leave Adjustment scenarios
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>2025-11-17</t>
+  </si>
+  <si>
+    <t>2025-11-18</t>
   </si>
 </sst>
 </file>
@@ -1265,7 +1268,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated HRM Locators and BOM locators
Updated HRM Locators and BOM locators
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>2025-12-04</t>
+  </si>
+  <si>
+    <t>2026-02-05</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1274,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Failed HRM module test scenarios
Fixed Failed HRM module test scenarios
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>2026-02-05</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
   </si>
 </sst>
 </file>
@@ -1274,7 +1277,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated HRM, POM test scenarios
Updated HRM, POM test scenarios
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>2026-07-09</t>
   </si>
 </sst>
 </file>
@@ -1277,7 +1283,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HRM module test scenarios fixes
HRM module test scenarios fixes
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>2026-07-09</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1286,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added and Updated Production module test scenarios
Added and Updated Production module test scenarios
</commit_message>
<xml_diff>
--- a/testdata/AccrualLeaveMigrationData.xlsx
+++ b/testdata/AccrualLeaveMigrationData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
   <si>
     <t>Emp.ID</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
   </si>
 </sst>
 </file>
@@ -1286,7 +1289,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>